<commit_message>
feat: added quality of life
</commit_message>
<xml_diff>
--- a/public/attendance-import-template.xlsx
+++ b/public/attendance-import-template.xlsx
@@ -9,6 +9,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D5"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="4" width="14" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -18,50 +23,90 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>2025-10-13</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2025-10-17</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>REPLACE_WITH_STUDENT_NUMBER_1</t>
+          <t>20260001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>P</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>REPLACE_WITH_STUDENT_NUMBER_2</t>
+          <t>20260002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>REPLACE_WITH_STUDENT_NUMBER_3</t>
+          <t>20260003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>Late</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Excused</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REPLACE_WITH_STUDENT_NUMBER_4</t>
+          <t>20260004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -69,6 +114,16 @@
           <t>E</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>